<commit_message>
Aktualizace dat z webové aplikace
</commit_message>
<xml_diff>
--- a/prohlidky.xlsx
+++ b/prohlidky.xlsx
@@ -421,27 +421,27 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Unnamed: 0</t>
+          <t>Číslo mašiny</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Datum provedení prohlídky a rozsah</t>
+          <t>Datum provedení</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Unnamed: 2</t>
+          <t>Provedena prohlídka</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Přístí prohlídka a rozsah</t>
+          <t>Příští prohlídka</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Unnamed: 4</t>
+          <t>Budoucí prohlídka</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">

</xml_diff>